<commit_message>
Update for May 2025 votes, change order of merge of pre-Tory resignation dataframe
</commit_message>
<xml_diff>
--- a/utils/similarity_chw.xlsx
+++ b/utils/similarity_chw.xlsx
@@ -19082,7 +19082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC29"/>
+  <dimension ref="A1:AD30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19148,14 +19148,14 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>Paula Fletcher</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Jennifer McKelvie</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Paula Fletcher</t>
-        </is>
-      </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Mike Colle</t>
@@ -19168,60 +19168,65 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
+          <t>Rachel Chernos Lin</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>Lily Cheng</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Frances Nunziata</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Anthony Perruzza</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>James Pasternak</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Nick Mantas</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Anthony Perruzza</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Jon Burnside</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>James Pasternak</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Jaye Robinson</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Brad Bradford</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Vincent Crisanti</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Stephen Holyday</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>John Tory</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Gary Crawford</t>
         </is>
@@ -19237,82 +19242,85 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9772727272727273</v>
+        <v>0.9814814814814815</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9767441860465116</v>
+        <v>0.9811320754716981</v>
       </c>
       <c r="E2" t="n">
-        <v>0.975</v>
+        <v>0.9795918367346939</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9696969696969697</v>
+        <v>0.9743589743589743</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9574468085106383</v>
+        <v>0.9649122807017544</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9565217391304348</v>
+        <v>0.9642857142857143</v>
       </c>
       <c r="I2" t="n">
-        <v>0.9565217391304348</v>
+        <v>0.9642857142857143</v>
       </c>
       <c r="J2" t="n">
-        <v>0.9361702127659575</v>
+        <v>0.9473684210526316</v>
       </c>
       <c r="K2" t="n">
-        <v>0.9361702127659575</v>
+        <v>0.9473684210526316</v>
       </c>
       <c r="L2" t="n">
-        <v>0.9361702127659575</v>
+        <v>0.9473684210526316</v>
       </c>
       <c r="M2" t="n">
-        <v>0.9361702127659575</v>
+        <v>0.9464285714285714</v>
       </c>
       <c r="N2" t="n">
-        <v>0.9302325581395349</v>
+        <v>0.9433962264150944</v>
       </c>
       <c r="O2" t="n">
-        <v>0.9302325581395349</v>
+        <v>0.92</v>
       </c>
       <c r="P2" t="n">
-        <v>0.8837209302325582</v>
+        <v>0.9038461538461539</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.8620689655172413</v>
+        <v>0.8717948717948718</v>
       </c>
       <c r="R2" t="n">
-        <v>0.8444444444444444</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="S2" t="n">
-        <v>0.8085106382978724</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="T2" t="n">
-        <v>0.7674418604651163</v>
+        <v>0.8245614035087719</v>
       </c>
       <c r="U2" t="n">
-        <v>0.7380952380952381</v>
+        <v>0.7307692307692308</v>
       </c>
       <c r="V2" t="n">
-        <v>0.717948717948718</v>
+        <v>0.7115384615384616</v>
       </c>
       <c r="W2" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.6923076923076923</v>
       </c>
       <c r="X2" t="n">
+        <v>0.6666666666666667</v>
+      </c>
+      <c r="Y2" t="n">
         <v>0.6086956521739131</v>
       </c>
-      <c r="Y2" t="n">
-        <v>0.5777777777777777</v>
-      </c>
       <c r="Z2" t="n">
-        <v>0.5151515151515151</v>
+        <v>0.5454545454545454</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.148936170212766</v>
-      </c>
-      <c r="AB2" t="inlineStr"/>
+        <v>0.5</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0.1228070175438597</v>
+      </c>
       <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -19321,87 +19329,90 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9772727272727273</v>
+        <v>0.9814814814814815</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.9310344827586207</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8913043478260869</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="F3" t="n">
-        <v>0.8205128205128205</v>
+        <v>0.8444444444444444</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9230769230769231</v>
+        <v>0.935483870967742</v>
       </c>
       <c r="H3" t="n">
-        <v>0.9215686274509804</v>
+        <v>0.9344262295081968</v>
       </c>
       <c r="I3" t="n">
-        <v>0.9607843137254902</v>
+        <v>0.9672131147540983</v>
       </c>
       <c r="J3" t="n">
-        <v>0.8823529411764706</v>
+        <v>0.9016393442622951</v>
       </c>
       <c r="K3" t="n">
-        <v>0.9230769230769231</v>
+        <v>0.935483870967742</v>
       </c>
       <c r="L3" t="n">
-        <v>0.9423076923076923</v>
+        <v>0.9516129032258065</v>
       </c>
       <c r="M3" t="n">
-        <v>0.9423076923076923</v>
+        <v>0.9508196721311475</v>
       </c>
       <c r="N3" t="n">
-        <v>0.8541666666666666</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="O3" t="n">
-        <v>0.92</v>
+        <v>0.8545454545454545</v>
       </c>
       <c r="P3" t="n">
-        <v>0.8541666666666666</v>
+        <v>0.8771929824561404</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.8918918918918919</v>
       </c>
       <c r="R3" t="n">
-        <v>0.84</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="S3" t="n">
-        <v>0.7307692307692308</v>
+        <v>0.8305084745762712</v>
       </c>
       <c r="T3" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.7580645161290323</v>
       </c>
       <c r="U3" t="n">
-        <v>0.6304347826086957</v>
+        <v>0.6428571428571428</v>
       </c>
       <c r="V3" t="n">
-        <v>0.6279069767441861</v>
+        <v>0.631578947368421</v>
       </c>
       <c r="W3" t="n">
-        <v>0.6170212765957447</v>
+        <v>0.6140350877192983</v>
       </c>
       <c r="X3" t="n">
+        <v>0.5961538461538461</v>
+      </c>
+      <c r="Y3" t="n">
         <v>0.5517241379310345</v>
       </c>
-      <c r="Y3" t="n">
-        <v>0.5490196078431373</v>
-      </c>
       <c r="Z3" t="n">
-        <v>0.4736842105263158</v>
+        <v>0.5245901639344263</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.1730769230769231</v>
+        <v>0.4680851063829787</v>
       </c>
       <c r="AB3" t="n">
+        <v>0.1451612903225806</v>
+      </c>
+      <c r="AC3" t="n">
         <v>0.5</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AD3" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -19412,87 +19423,90 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9767441860465116</v>
+        <v>0.9811320754716981</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.9310344827586207</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="n">
+        <v>0.9433962264150944</v>
+      </c>
+      <c r="F4" t="n">
         <v>0.9318181818181819</v>
       </c>
-      <c r="F4" t="n">
-        <v>0.9210526315789473</v>
-      </c>
       <c r="G4" t="n">
-        <v>0.8431372549019608</v>
+        <v>0.8688524590163934</v>
       </c>
       <c r="H4" t="n">
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
       <c r="I4" t="n">
-        <v>0.86</v>
+        <v>0.8833333333333333</v>
       </c>
       <c r="J4" t="n">
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
       <c r="K4" t="n">
-        <v>0.8431372549019608</v>
+        <v>0.8688524590163934</v>
       </c>
       <c r="L4" t="n">
-        <v>0.8431372549019608</v>
+        <v>0.8688524590163934</v>
       </c>
       <c r="M4" t="n">
-        <v>0.8431372549019608</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="N4" t="n">
-        <v>0.9574468085106383</v>
+        <v>0.8596491228070176</v>
       </c>
       <c r="O4" t="n">
-        <v>0.8297872340425532</v>
+        <v>0.9444444444444444</v>
       </c>
       <c r="P4" t="n">
-        <v>0.8297872340425532</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.92</v>
+        <v>0.9142857142857143</v>
       </c>
       <c r="R4" t="n">
-        <v>0.8367346938775511</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="S4" t="n">
-        <v>0.8235294117647058</v>
+        <v>0.8275862068965517</v>
       </c>
       <c r="T4" t="n">
-        <v>0.75</v>
+        <v>0.8360655737704918</v>
       </c>
       <c r="U4" t="n">
+        <v>0.6181818181818182</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.6964285714285714</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.6842105263157895</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0.607843137254902</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0.5862068965517242</v>
+      </c>
+      <c r="Z4" t="n">
         <v>0.6</v>
       </c>
-      <c r="V4" t="n">
-        <v>0.6428571428571428</v>
-      </c>
-      <c r="W4" t="n">
-        <v>0.6956521739130435</v>
-      </c>
-      <c r="X4" t="n">
-        <v>0.5862068965517242</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>0.5526315789473684</v>
-      </c>
       <c r="AA4" t="n">
-        <v>0.2156862745098039</v>
+        <v>0.5319148936170213</v>
       </c>
       <c r="AB4" t="n">
+        <v>0.180327868852459</v>
+      </c>
+      <c r="AC4" t="n">
         <v>0.875</v>
       </c>
-      <c r="AC4" t="n">
+      <c r="AD4" t="n">
         <v>0.875</v>
       </c>
     </row>
@@ -19503,87 +19517,90 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.975</v>
+        <v>0.9795918367346939</v>
       </c>
       <c r="C5" t="n">
-        <v>0.8913043478260869</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9318181818181819</v>
+        <v>0.9433962264150944</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9</v>
+        <v>0.9130434782608696</v>
       </c>
       <c r="G5" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.8596491228070176</v>
       </c>
       <c r="H5" t="n">
-        <v>0.8936170212765957</v>
+        <v>0.9107142857142857</v>
       </c>
       <c r="I5" t="n">
-        <v>0.8723404255319149</v>
+        <v>0.8928571428571429</v>
       </c>
       <c r="J5" t="n">
-        <v>0.851063829787234</v>
+        <v>0.875</v>
       </c>
       <c r="K5" t="n">
-        <v>0.8541666666666666</v>
+        <v>0.8771929824561404</v>
       </c>
       <c r="L5" t="n">
-        <v>0.8541666666666666</v>
+        <v>0.8771929824561404</v>
       </c>
       <c r="M5" t="n">
-        <v>0.8541666666666666</v>
+        <v>0.8771929824561404</v>
       </c>
       <c r="N5" t="n">
-        <v>0.8863636363636364</v>
+        <v>0.8679245283018868</v>
       </c>
       <c r="O5" t="n">
-        <v>0.8409090909090909</v>
+        <v>0.8823529411764706</v>
       </c>
       <c r="P5" t="n">
-        <v>0.8444444444444444</v>
+        <v>0.8703703703703703</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.9230769230769231</v>
+        <v>0.9142857142857143</v>
       </c>
       <c r="R5" t="n">
-        <v>0.7826086956521739</v>
+        <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>0.75</v>
+        <v>0.7962962962962963</v>
       </c>
       <c r="T5" t="n">
-        <v>0.75</v>
+        <v>0.7894736842105263</v>
       </c>
       <c r="U5" t="n">
-        <v>0.6818181818181819</v>
+        <v>0.6981132075471699</v>
       </c>
       <c r="V5" t="n">
         <v>0.6666666666666667</v>
       </c>
       <c r="W5" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.6923076923076923</v>
       </c>
       <c r="X5" t="n">
+        <v>0.6382978723404256</v>
+      </c>
+      <c r="Y5" t="n">
         <v>0.6538461538461539</v>
       </c>
-      <c r="Y5" t="n">
-        <v>0.6170212765957447</v>
-      </c>
       <c r="Z5" t="n">
-        <v>0.5277777777777778</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.2708333333333334</v>
+        <v>0.5</v>
       </c>
       <c r="AB5" t="n">
+        <v>0.2280701754385965</v>
+      </c>
+      <c r="AC5" t="n">
         <v>0.625</v>
       </c>
-      <c r="AC5" t="n">
+      <c r="AD5" t="n">
         <v>0.625</v>
       </c>
     </row>
@@ -19594,87 +19611,90 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.9696969696969697</v>
+        <v>0.9743589743589743</v>
       </c>
       <c r="C6" t="n">
-        <v>0.8205128205128205</v>
+        <v>0.8444444444444444</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9210526315789473</v>
+        <v>0.9318181818181819</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9</v>
+        <v>0.9130434782608696</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>0.7560975609756098</v>
+        <v>0.7872340425531915</v>
       </c>
       <c r="H6" t="n">
-        <v>0.8</v>
+        <v>0.8260869565217391</v>
       </c>
       <c r="I6" t="n">
-        <v>0.75</v>
+        <v>0.7826086956521739</v>
       </c>
       <c r="J6" t="n">
-        <v>0.8</v>
+        <v>0.8260869565217391</v>
       </c>
       <c r="K6" t="n">
-        <v>0.7317073170731707</v>
+        <v>0.7659574468085106</v>
       </c>
       <c r="L6" t="n">
-        <v>0.7317073170731707</v>
+        <v>0.7659574468085106</v>
       </c>
       <c r="M6" t="n">
-        <v>0.7317073170731707</v>
+        <v>0.7659574468085106</v>
       </c>
       <c r="N6" t="n">
-        <v>0.8918918918918919</v>
+        <v>0.7441860465116279</v>
       </c>
       <c r="O6" t="n">
-        <v>0.7027027027027026</v>
+        <v>0.8780487804878049</v>
       </c>
       <c r="P6" t="n">
-        <v>0.7894736842105263</v>
+        <v>0.8181818181818181</v>
       </c>
       <c r="Q6" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="R6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.7111111111111111</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.8936170212765957</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.6511627906976745</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.7045454545454546</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.8181818181818181</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0.7105263157894737</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0.6818181818181819</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0.6382978723404256</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>0.2340425531914894</v>
+      </c>
+      <c r="AC6" t="n">
         <v>0.875</v>
       </c>
-      <c r="R6" t="n">
-        <v>0.6923076923076923</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0.8780487804878049</v>
-      </c>
-      <c r="T6" t="n">
-        <v>0.8717948717948718</v>
-      </c>
-      <c r="U6" t="n">
-        <v>0.6486486486486487</v>
-      </c>
-      <c r="V6" t="n">
-        <v>0.7272727272727273</v>
-      </c>
-      <c r="W6" t="n">
-        <v>0.736842105263158</v>
-      </c>
-      <c r="X6" t="n">
-        <v>0.6818181818181819</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>0.6829268292682926</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>0.6666666666666667</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>0.2682926829268293</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="AC6" t="n">
+      <c r="AD6" t="n">
         <v>0.875</v>
       </c>
     </row>
@@ -19685,87 +19705,90 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.9574468085106383</v>
+        <v>0.9649122807017544</v>
       </c>
       <c r="C7" t="n">
-        <v>0.9230769230769231</v>
+        <v>0.935483870967742</v>
       </c>
       <c r="D7" t="n">
-        <v>0.8431372549019608</v>
+        <v>0.8688524590163934</v>
       </c>
       <c r="E7" t="n">
+        <v>0.8596491228070176</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.7872340425531915</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.921875</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.96875</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.9538461538461538</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.9846153846153847</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.984375</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.9672131147540983</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.8103448275862069</v>
+      </c>
+      <c r="P7" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="F7" t="n">
-        <v>0.7560975609756098</v>
-      </c>
-      <c r="G7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.9074074074074074</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.962962962962963</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0.9259259259259259</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0.9454545454545454</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.9818181818181818</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0.9818181818181818</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0.803921568627451</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0.9607843137254902</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0.803921568627451</v>
-      </c>
       <c r="Q7" t="n">
-        <v>0.7931034482758621</v>
+        <v>0.8205128205128205</v>
       </c>
       <c r="R7" t="n">
-        <v>0.8490566037735849</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="S7" t="n">
-        <v>0.6909090909090909</v>
+        <v>0.8387096774193549</v>
       </c>
       <c r="T7" t="n">
-        <v>0.6274509803921569</v>
+        <v>0.7230769230769231</v>
       </c>
       <c r="U7" t="n">
-        <v>0.653061224489796</v>
+        <v>0.6610169491525424</v>
       </c>
       <c r="V7" t="n">
-        <v>0.5652173913043479</v>
+        <v>0.6</v>
       </c>
       <c r="W7" t="n">
-        <v>0.5800000000000001</v>
+        <v>0.5833333333333333</v>
       </c>
       <c r="X7" t="n">
+        <v>0.5454545454545454</v>
+      </c>
+      <c r="Y7" t="n">
         <v>0.5517241379310345</v>
       </c>
-      <c r="Y7" t="n">
-        <v>0.5094339622641509</v>
-      </c>
       <c r="Z7" t="n">
-        <v>0.4146341463414634</v>
+        <v>0.4920634920634921</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.1454545454545455</v>
+        <v>0.42</v>
       </c>
       <c r="AB7" t="n">
+        <v>0.1230769230769231</v>
+      </c>
+      <c r="AC7" t="n">
         <v>0.25</v>
       </c>
-      <c r="AC7" t="n">
+      <c r="AD7" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -19776,87 +19799,90 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.9565217391304348</v>
+        <v>0.9642857142857143</v>
       </c>
       <c r="C8" t="n">
-        <v>0.9215686274509804</v>
+        <v>0.9344262295081968</v>
       </c>
       <c r="D8" t="n">
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
       <c r="E8" t="n">
-        <v>0.8936170212765957</v>
+        <v>0.9107142857142857</v>
       </c>
       <c r="F8" t="n">
-        <v>0.8</v>
+        <v>0.8260869565217391</v>
       </c>
       <c r="G8" t="n">
-        <v>0.9074074074074074</v>
+        <v>0.921875</v>
       </c>
       <c r="H8" t="n">
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>0.9433962264150944</v>
+        <v>0.9523809523809523</v>
       </c>
       <c r="J8" t="n">
-        <v>0.8867924528301887</v>
+        <v>0.9047619047619048</v>
       </c>
       <c r="K8" t="n">
-        <v>0.9259259259259259</v>
+        <v>0.9375</v>
       </c>
       <c r="L8" t="n">
-        <v>0.9259259259259259</v>
+        <v>0.9375</v>
       </c>
       <c r="M8" t="n">
-        <v>0.9259259259259259</v>
+        <v>0.9365079365079365</v>
       </c>
       <c r="N8" t="n">
-        <v>0.8200000000000001</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="O8" t="n">
-        <v>0.92</v>
+        <v>0.8245614035087719</v>
       </c>
       <c r="P8" t="n">
-        <v>0.8200000000000001</v>
+        <v>0.847457627118644</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.8928571428571429</v>
+        <v>0.8947368421052632</v>
       </c>
       <c r="R8" t="n">
-        <v>0.8679245283018868</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="S8" t="n">
-        <v>0.7407407407407407</v>
+        <v>0.8548387096774194</v>
       </c>
       <c r="T8" t="n">
-        <v>0.6799999999999999</v>
+        <v>0.765625</v>
       </c>
       <c r="U8" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.6724137931034483</v>
       </c>
       <c r="V8" t="n">
-        <v>0.6</v>
+        <v>0.6101694915254237</v>
       </c>
       <c r="W8" t="n">
-        <v>0.5918367346938775</v>
+        <v>0.6271186440677966</v>
       </c>
       <c r="X8" t="n">
+        <v>0.5740740740740741</v>
+      </c>
+      <c r="Y8" t="n">
         <v>0.5172413793103448</v>
       </c>
-      <c r="Y8" t="n">
-        <v>0.5576923076923077</v>
-      </c>
       <c r="Z8" t="n">
-        <v>0.4878048780487805</v>
+        <v>0.532258064516129</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.2407407407407407</v>
+        <v>0.48</v>
       </c>
       <c r="AB8" t="n">
+        <v>0.203125</v>
+      </c>
+      <c r="AC8" t="n">
         <v>0.375</v>
       </c>
-      <c r="AC8" t="n">
+      <c r="AD8" t="n">
         <v>0.375</v>
       </c>
     </row>
@@ -19867,87 +19893,90 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.9565217391304348</v>
+        <v>0.9642857142857143</v>
       </c>
       <c r="C9" t="n">
-        <v>0.9607843137254902</v>
+        <v>0.9672131147540983</v>
       </c>
       <c r="D9" t="n">
-        <v>0.86</v>
+        <v>0.8833333333333333</v>
       </c>
       <c r="E9" t="n">
-        <v>0.8723404255319149</v>
+        <v>0.8928571428571429</v>
       </c>
       <c r="F9" t="n">
-        <v>0.75</v>
+        <v>0.7826086956521739</v>
       </c>
       <c r="G9" t="n">
-        <v>0.962962962962963</v>
+        <v>0.96875</v>
       </c>
       <c r="H9" t="n">
-        <v>0.9433962264150944</v>
+        <v>0.9523809523809523</v>
       </c>
       <c r="I9" t="n">
         <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0.9245283018867925</v>
+        <v>0.9365079365079365</v>
       </c>
       <c r="K9" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.953125</v>
       </c>
       <c r="L9" t="n">
-        <v>0.9814814814814815</v>
+        <v>0.984375</v>
       </c>
       <c r="M9" t="n">
-        <v>0.9814814814814815</v>
+        <v>0.9841269841269842</v>
       </c>
       <c r="N9" t="n">
-        <v>0.8</v>
+        <v>0.9666666666666667</v>
       </c>
       <c r="O9" t="n">
-        <v>0.96</v>
+        <v>0.8070175438596492</v>
       </c>
       <c r="P9" t="n">
-        <v>0.803921568627451</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="Q9" t="n">
+        <v>0.868421052631579</v>
+      </c>
+      <c r="R9" t="n">
         <v>0.8571428571428572</v>
       </c>
-      <c r="R9" t="n">
-        <v>0.8846153846153846</v>
-      </c>
       <c r="S9" t="n">
-        <v>0.6851851851851851</v>
+        <v>0.8688524590163934</v>
       </c>
       <c r="T9" t="n">
-        <v>0.62</v>
+        <v>0.71875</v>
       </c>
       <c r="U9" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.6724137931034483</v>
       </c>
       <c r="V9" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.6</v>
       </c>
       <c r="W9" t="n">
-        <v>0.5800000000000001</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="X9" t="n">
+        <v>0.537037037037037</v>
+      </c>
+      <c r="Y9" t="n">
         <v>0.5862068965517242</v>
       </c>
-      <c r="Y9" t="n">
-        <v>0.5</v>
-      </c>
       <c r="Z9" t="n">
-        <v>0.4146341463414634</v>
+        <v>0.4838709677419355</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.1666666666666666</v>
+        <v>0.42</v>
       </c>
       <c r="AB9" t="n">
+        <v>0.140625</v>
+      </c>
+      <c r="AC9" t="n">
         <v>0.25</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="AD9" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -19958,87 +19987,90 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.9361702127659575</v>
+        <v>0.9473684210526316</v>
       </c>
       <c r="C10" t="n">
-        <v>0.8823529411764706</v>
+        <v>0.9016393442622951</v>
       </c>
       <c r="D10" t="n">
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
       <c r="E10" t="n">
-        <v>0.851063829787234</v>
+        <v>0.875</v>
       </c>
       <c r="F10" t="n">
-        <v>0.8</v>
+        <v>0.8260869565217391</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9259259259259259</v>
+        <v>0.9375</v>
       </c>
       <c r="H10" t="n">
-        <v>0.8867924528301887</v>
+        <v>0.9047619047619048</v>
       </c>
       <c r="I10" t="n">
-        <v>0.9245283018867925</v>
+        <v>0.9365079365079365</v>
       </c>
       <c r="J10" t="n">
         <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>0.8703703703703703</v>
+        <v>0.890625</v>
       </c>
       <c r="L10" t="n">
-        <v>0.9074074074074074</v>
+        <v>0.921875</v>
       </c>
       <c r="M10" t="n">
-        <v>0.9074074074074074</v>
+        <v>0.9206349206349207</v>
       </c>
       <c r="N10" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="O10" t="n">
-        <v>0.88</v>
+        <v>0.8596491228070176</v>
       </c>
       <c r="P10" t="n">
-        <v>0.8200000000000001</v>
+        <v>0.847457627118644</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.7586206896551724</v>
+        <v>0.7948717948717949</v>
       </c>
       <c r="R10" t="n">
-        <v>0.8653846153846154</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="S10" t="n">
-        <v>0.7407407407407407</v>
+        <v>0.8524590163934427</v>
       </c>
       <c r="T10" t="n">
-        <v>0.6799999999999999</v>
+        <v>0.765625</v>
       </c>
       <c r="U10" t="n">
-        <v>0.625</v>
+        <v>0.6379310344827587</v>
       </c>
       <c r="V10" t="n">
-        <v>0.6222222222222222</v>
+        <v>0.6440677966101696</v>
       </c>
       <c r="W10" t="n">
-        <v>0.6326530612244898</v>
+        <v>0.6271186440677966</v>
       </c>
       <c r="X10" t="n">
+        <v>0.5925925925925926</v>
+      </c>
+      <c r="Y10" t="n">
         <v>0.5714285714285714</v>
       </c>
-      <c r="Y10" t="n">
-        <v>0.5576923076923077</v>
-      </c>
       <c r="Z10" t="n">
-        <v>0.475</v>
+        <v>0.532258064516129</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.4693877551020408</v>
       </c>
       <c r="AB10" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="AC10" t="n">
         <v>0.4285714285714286</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="AD10" t="n">
         <v>0.4285714285714286</v>
       </c>
     </row>
@@ -20049,87 +20081,90 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.9361702127659575</v>
+        <v>0.9473684210526316</v>
       </c>
       <c r="C11" t="n">
-        <v>0.9230769230769231</v>
+        <v>0.935483870967742</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8431372549019608</v>
+        <v>0.8688524590163934</v>
       </c>
       <c r="E11" t="n">
-        <v>0.8541666666666666</v>
+        <v>0.8771929824561404</v>
       </c>
       <c r="F11" t="n">
-        <v>0.7317073170731707</v>
+        <v>0.7659574468085106</v>
       </c>
       <c r="G11" t="n">
-        <v>0.9454545454545454</v>
+        <v>0.9538461538461538</v>
       </c>
       <c r="H11" t="n">
-        <v>0.9259259259259259</v>
+        <v>0.9375</v>
       </c>
       <c r="I11" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.953125</v>
       </c>
       <c r="J11" t="n">
-        <v>0.8703703703703703</v>
+        <v>0.890625</v>
       </c>
       <c r="K11" t="n">
         <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>0.9636363636363636</v>
+        <v>0.9692307692307692</v>
       </c>
       <c r="M11" t="n">
-        <v>0.9636363636363636</v>
+        <v>0.96875</v>
       </c>
       <c r="N11" t="n">
-        <v>0.7843137254901961</v>
+        <v>0.9672131147540983</v>
       </c>
       <c r="O11" t="n">
-        <v>0.9607843137254902</v>
+        <v>0.7931034482758621</v>
       </c>
       <c r="P11" t="n">
-        <v>0.8235294117647058</v>
+        <v>0.85</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.8275862068965517</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="R11" t="n">
-        <v>0.8301886792452831</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="S11" t="n">
-        <v>0.6727272727272727</v>
+        <v>0.8225806451612903</v>
       </c>
       <c r="T11" t="n">
-        <v>0.607843137254902</v>
+        <v>0.7076923076923076</v>
       </c>
       <c r="U11" t="n">
-        <v>0.6326530612244898</v>
+        <v>0.6440677966101696</v>
       </c>
       <c r="V11" t="n">
-        <v>0.5652173913043479</v>
+        <v>0.5833333333333333</v>
       </c>
       <c r="W11" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="X11" t="n">
+        <v>0.5454545454545454</v>
+      </c>
+      <c r="Y11" t="n">
         <v>0.5172413793103448</v>
       </c>
-      <c r="Y11" t="n">
-        <v>0.4905660377358491</v>
-      </c>
       <c r="Z11" t="n">
-        <v>0.4146341463414634</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.2</v>
+        <v>0.42</v>
       </c>
       <c r="AB11" t="n">
+        <v>0.1692307692307692</v>
+      </c>
+      <c r="AC11" t="n">
         <v>0.25</v>
       </c>
-      <c r="AC11" t="n">
+      <c r="AD11" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -20140,34 +20175,34 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.9361702127659575</v>
+        <v>0.9473684210526316</v>
       </c>
       <c r="C12" t="n">
-        <v>0.9423076923076923</v>
+        <v>0.9516129032258065</v>
       </c>
       <c r="D12" t="n">
-        <v>0.8431372549019608</v>
+        <v>0.8688524590163934</v>
       </c>
       <c r="E12" t="n">
-        <v>0.8541666666666666</v>
+        <v>0.8771929824561404</v>
       </c>
       <c r="F12" t="n">
-        <v>0.7317073170731707</v>
+        <v>0.7659574468085106</v>
       </c>
       <c r="G12" t="n">
-        <v>0.9818181818181818</v>
+        <v>0.9846153846153847</v>
       </c>
       <c r="H12" t="n">
-        <v>0.9259259259259259</v>
+        <v>0.9375</v>
       </c>
       <c r="I12" t="n">
-        <v>0.9814814814814815</v>
+        <v>0.984375</v>
       </c>
       <c r="J12" t="n">
-        <v>0.9074074074074074</v>
+        <v>0.921875</v>
       </c>
       <c r="K12" t="n">
-        <v>0.9636363636363636</v>
+        <v>0.9692307692307692</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -20176,51 +20211,54 @@
         <v>1</v>
       </c>
       <c r="N12" t="n">
-        <v>0.7843137254901961</v>
+        <v>0.9836065573770492</v>
       </c>
       <c r="O12" t="n">
-        <v>0.9803921568627451</v>
+        <v>0.7931034482758621</v>
       </c>
       <c r="P12" t="n">
-        <v>0.7843137254901961</v>
+        <v>0.8166666666666667</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.8275862068965517</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="R12" t="n">
-        <v>0.8679245283018868</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="S12" t="n">
-        <v>0.6727272727272727</v>
+        <v>0.8548387096774194</v>
       </c>
       <c r="T12" t="n">
-        <v>0.607843137254902</v>
+        <v>0.7076923076923076</v>
       </c>
       <c r="U12" t="n">
-        <v>0.6326530612244898</v>
+        <v>0.6440677966101696</v>
       </c>
       <c r="V12" t="n">
-        <v>0.5434782608695652</v>
+        <v>0.5833333333333333</v>
       </c>
       <c r="W12" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="X12" t="n">
+        <v>0.5272727272727273</v>
+      </c>
+      <c r="Y12" t="n">
         <v>0.5517241379310345</v>
       </c>
-      <c r="Y12" t="n">
-        <v>0.4905660377358491</v>
-      </c>
       <c r="Z12" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.1636363636363637</v>
+        <v>0.4</v>
       </c>
       <c r="AB12" t="n">
+        <v>0.1384615384615384</v>
+      </c>
+      <c r="AC12" t="n">
         <v>0.25</v>
       </c>
-      <c r="AC12" t="n">
+      <c r="AD12" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -20231,34 +20269,34 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.9361702127659575</v>
+        <v>0.9464285714285714</v>
       </c>
       <c r="C13" t="n">
-        <v>0.9423076923076923</v>
+        <v>0.9508196721311475</v>
       </c>
       <c r="D13" t="n">
-        <v>0.8431372549019608</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="E13" t="n">
-        <v>0.8541666666666666</v>
+        <v>0.8771929824561404</v>
       </c>
       <c r="F13" t="n">
-        <v>0.7317073170731707</v>
+        <v>0.7659574468085106</v>
       </c>
       <c r="G13" t="n">
-        <v>0.9818181818181818</v>
+        <v>0.984375</v>
       </c>
       <c r="H13" t="n">
-        <v>0.9259259259259259</v>
+        <v>0.9365079365079365</v>
       </c>
       <c r="I13" t="n">
-        <v>0.9814814814814815</v>
+        <v>0.9841269841269842</v>
       </c>
       <c r="J13" t="n">
-        <v>0.9074074074074074</v>
+        <v>0.9206349206349207</v>
       </c>
       <c r="K13" t="n">
-        <v>0.9636363636363636</v>
+        <v>0.96875</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -20267,234 +20305,243 @@
         <v>1</v>
       </c>
       <c r="N13" t="n">
-        <v>0.7843137254901961</v>
+        <v>0.9833333333333333</v>
       </c>
       <c r="O13" t="n">
-        <v>0.9803921568627451</v>
+        <v>0.7931034482758621</v>
       </c>
       <c r="P13" t="n">
-        <v>0.7843137254901961</v>
+        <v>0.8166666666666667</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.8275862068965517</v>
+        <v>0.8421052631578947</v>
       </c>
       <c r="R13" t="n">
-        <v>0.8679245283018868</v>
+        <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>0.6727272727272727</v>
+        <v>0.8688524590163934</v>
       </c>
       <c r="T13" t="n">
-        <v>0.607843137254902</v>
+        <v>0.71875</v>
       </c>
       <c r="U13" t="n">
-        <v>0.6326530612244898</v>
+        <v>0.6551724137931034</v>
       </c>
       <c r="V13" t="n">
-        <v>0.5434782608695652</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="W13" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="X13" t="n">
+        <v>0.537037037037037</v>
+      </c>
+      <c r="Y13" t="n">
         <v>0.5517241379310345</v>
       </c>
-      <c r="Y13" t="n">
-        <v>0.4905660377358491</v>
-      </c>
       <c r="Z13" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.467741935483871</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.1636363636363637</v>
+        <v>0.3877551020408163</v>
       </c>
       <c r="AB13" t="n">
+        <v>0.140625</v>
+      </c>
+      <c r="AC13" t="n">
         <v>0.25</v>
       </c>
-      <c r="AC13" t="n">
+      <c r="AD13" t="n">
         <v>0.25</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>Jennifer McKelvie</t>
+          <t>Paula Fletcher</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.9302325581395349</v>
+        <v>0.9433962264150944</v>
       </c>
       <c r="C14" t="n">
-        <v>0.8541666666666666</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="D14" t="n">
-        <v>0.9574468085106383</v>
+        <v>0.8596491228070176</v>
       </c>
       <c r="E14" t="n">
-        <v>0.8863636363636364</v>
+        <v>0.8679245283018868</v>
       </c>
       <c r="F14" t="n">
-        <v>0.8918918918918919</v>
+        <v>0.7441860465116279</v>
       </c>
       <c r="G14" t="n">
-        <v>0.803921568627451</v>
+        <v>0.9672131147540983</v>
       </c>
       <c r="H14" t="n">
-        <v>0.8200000000000001</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="I14" t="n">
-        <v>0.8</v>
+        <v>0.9666666666666667</v>
       </c>
       <c r="J14" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="K14" t="n">
-        <v>0.7843137254901961</v>
+        <v>0.9672131147540983</v>
       </c>
       <c r="L14" t="n">
-        <v>0.7843137254901961</v>
+        <v>0.9836065573770492</v>
       </c>
       <c r="M14" t="n">
-        <v>0.7843137254901961</v>
+        <v>0.9833333333333333</v>
       </c>
       <c r="N14" t="n">
         <v>1</v>
       </c>
       <c r="O14" t="n">
-        <v>0.7659574468085106</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="P14" t="n">
-        <v>0.8297872340425532</v>
+        <v>0.8214285714285714</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.7692307692307692</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="R14" t="n">
-        <v>0.7959183673469388</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="S14" t="n">
-        <v>0.8431372549019608</v>
+        <v>0.864406779661017</v>
       </c>
       <c r="T14" t="n">
-        <v>0.7872340425531915</v>
+        <v>0.6885245901639344</v>
       </c>
       <c r="U14" t="n">
-        <v>0.6086956521739131</v>
+        <v>0.6545454545454545</v>
       </c>
       <c r="V14" t="n">
-        <v>0.6904761904761905</v>
+        <v>0.5614035087719298</v>
       </c>
       <c r="W14" t="n">
-        <v>0.7391304347826086</v>
+        <v>0.5535714285714286</v>
       </c>
       <c r="X14" t="n">
-        <v>0.6071428571428572</v>
+        <v>0.5490196078431373</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.5</v>
       </c>
       <c r="Z14" t="n">
-        <v>0.631578947368421</v>
+        <v>0.4576271186440678</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.2745098039215687</v>
+        <v>0.3913043478260869</v>
       </c>
       <c r="AB14" t="n">
-        <v>0.875</v>
+        <v>0.1639344262295082</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.875</v>
+        <v>0.25</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>0.25</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>Paula Fletcher</t>
+          <t>Jennifer McKelvie</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.9302325581395349</v>
+        <v>0.92</v>
       </c>
       <c r="C15" t="n">
-        <v>0.92</v>
+        <v>0.8545454545454545</v>
       </c>
       <c r="D15" t="n">
-        <v>0.8297872340425532</v>
+        <v>0.9444444444444444</v>
       </c>
       <c r="E15" t="n">
-        <v>0.8409090909090909</v>
+        <v>0.8823529411764706</v>
       </c>
       <c r="F15" t="n">
-        <v>0.7027027027027026</v>
+        <v>0.8780487804878049</v>
       </c>
       <c r="G15" t="n">
-        <v>0.9607843137254902</v>
+        <v>0.8103448275862069</v>
       </c>
       <c r="H15" t="n">
-        <v>0.92</v>
+        <v>0.8245614035087719</v>
       </c>
       <c r="I15" t="n">
-        <v>0.96</v>
+        <v>0.8070175438596492</v>
       </c>
       <c r="J15" t="n">
-        <v>0.88</v>
+        <v>0.8596491228070176</v>
       </c>
       <c r="K15" t="n">
-        <v>0.9607843137254902</v>
+        <v>0.7931034482758621</v>
       </c>
       <c r="L15" t="n">
-        <v>0.9803921568627451</v>
+        <v>0.7931034482758621</v>
       </c>
       <c r="M15" t="n">
-        <v>0.9803921568627451</v>
+        <v>0.7931034482758621</v>
       </c>
       <c r="N15" t="n">
-        <v>0.7659574468085106</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="O15" t="n">
         <v>1</v>
       </c>
       <c r="P15" t="n">
-        <v>0.7872340425531915</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.84</v>
+        <v>0.8181818181818181</v>
       </c>
       <c r="R15" t="n">
-        <v>0.88</v>
+        <v>1</v>
       </c>
       <c r="S15" t="n">
-        <v>0.6470588235294117</v>
+        <v>0.7818181818181819</v>
       </c>
       <c r="T15" t="n">
-        <v>0.5957446808510638</v>
+        <v>0.8448275862068966</v>
       </c>
       <c r="U15" t="n">
-        <v>0.6444444444444444</v>
+        <v>0.6226415094339622</v>
       </c>
       <c r="V15" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.7547169811320755</v>
       </c>
       <c r="W15" t="n">
-        <v>0.5319148936170213</v>
+        <v>0.7735849056603774</v>
       </c>
       <c r="X15" t="n">
-        <v>0.5</v>
+        <v>0.6734693877551021</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.4693877551020408</v>
+        <v>0.6071428571428572</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.3783783783783784</v>
+        <v>0.6964285714285714</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.196078431372549</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="AB15" t="n">
-        <v>0.25</v>
+        <v>0.2586206896551724</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.25</v>
+        <v>0.875</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>0.875</v>
       </c>
     </row>
     <row r="16">
@@ -20504,87 +20551,90 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.8837209302325582</v>
+        <v>0.9038461538461539</v>
       </c>
       <c r="C16" t="n">
-        <v>0.8541666666666666</v>
+        <v>0.8771929824561404</v>
       </c>
       <c r="D16" t="n">
-        <v>0.8297872340425532</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="E16" t="n">
-        <v>0.8444444444444444</v>
+        <v>0.8703703703703703</v>
       </c>
       <c r="F16" t="n">
-        <v>0.7894736842105263</v>
+        <v>0.8181818181818181</v>
       </c>
       <c r="G16" t="n">
-        <v>0.803921568627451</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="H16" t="n">
-        <v>0.8200000000000001</v>
+        <v>0.847457627118644</v>
       </c>
       <c r="I16" t="n">
-        <v>0.803921568627451</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="J16" t="n">
-        <v>0.8200000000000001</v>
+        <v>0.847457627118644</v>
       </c>
       <c r="K16" t="n">
-        <v>0.8235294117647058</v>
+        <v>0.85</v>
       </c>
       <c r="L16" t="n">
-        <v>0.7843137254901961</v>
+        <v>0.8166666666666667</v>
       </c>
       <c r="M16" t="n">
-        <v>0.7843137254901961</v>
+        <v>0.8166666666666667</v>
       </c>
       <c r="N16" t="n">
-        <v>0.8297872340425532</v>
+        <v>0.8214285714285714</v>
       </c>
       <c r="O16" t="n">
-        <v>0.7872340425531915</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="P16" t="n">
         <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.6923076923076923</v>
+        <v>0.7428571428571429</v>
       </c>
       <c r="R16" t="n">
-        <v>0.7551020408163265</v>
+        <v>1</v>
       </c>
       <c r="S16" t="n">
-        <v>0.7254901960784313</v>
+        <v>0.7719298245614035</v>
       </c>
       <c r="T16" t="n">
-        <v>0.6595744680851063</v>
+        <v>0.7666666666666666</v>
       </c>
       <c r="U16" t="n">
-        <v>0.6</v>
+        <v>0.6296296296296297</v>
       </c>
       <c r="V16" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.6071428571428572</v>
       </c>
       <c r="W16" t="n">
-        <v>0.5957446808510638</v>
+        <v>0.6181818181818182</v>
       </c>
       <c r="X16" t="n">
+        <v>0.6799999999999999</v>
+      </c>
+      <c r="Y16" t="n">
         <v>0.5357142857142857</v>
       </c>
-      <c r="Y16" t="n">
-        <v>0.5918367346938775</v>
-      </c>
       <c r="Z16" t="n">
-        <v>0.5526315789473684</v>
+        <v>0.5517241379310345</v>
       </c>
       <c r="AA16" t="n">
-        <v>0.2941176470588235</v>
+        <v>0.5217391304347826</v>
       </c>
       <c r="AB16" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AC16" t="n">
         <v>0.625</v>
       </c>
-      <c r="AC16" t="n">
+      <c r="AD16" t="n">
         <v>0.625</v>
       </c>
     </row>
@@ -20595,357 +20645,363 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.8620689655172413</v>
+        <v>0.8717948717948718</v>
       </c>
       <c r="C17" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.8918918918918919</v>
       </c>
       <c r="D17" t="n">
-        <v>0.92</v>
+        <v>0.9142857142857143</v>
       </c>
       <c r="E17" t="n">
-        <v>0.9230769230769231</v>
+        <v>0.9142857142857143</v>
       </c>
       <c r="F17" t="n">
-        <v>0.875</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="G17" t="n">
-        <v>0.7931034482758621</v>
+        <v>0.8205128205128205</v>
       </c>
       <c r="H17" t="n">
-        <v>0.8928571428571429</v>
+        <v>0.8947368421052632</v>
       </c>
       <c r="I17" t="n">
+        <v>0.868421052631579</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.7948717948717949</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.8421052631578947</v>
+      </c>
+      <c r="N17" t="n">
         <v>0.8571428571428572</v>
       </c>
-      <c r="J17" t="n">
-        <v>0.7586206896551724</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0.8275862068965517</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0.8275862068965517</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0.8275862068965517</v>
-      </c>
-      <c r="N17" t="n">
-        <v>0.7692307692307692</v>
-      </c>
       <c r="O17" t="n">
-        <v>0.84</v>
+        <v>0.8181818181818181</v>
       </c>
       <c r="P17" t="n">
-        <v>0.6923076923076923</v>
+        <v>0.7428571428571429</v>
       </c>
       <c r="Q17" t="n">
         <v>1</v>
       </c>
       <c r="R17" t="n">
-        <v>0.8518518518518519</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="S17" t="n">
-        <v>0.8275862068965517</v>
+        <v>0.8055555555555556</v>
       </c>
       <c r="T17" t="n">
-        <v>0.7037037037037037</v>
+        <v>0.8205128205128205</v>
       </c>
       <c r="U17" t="n">
-        <v>0.7083333333333333</v>
+        <v>0.6764705882352942</v>
       </c>
       <c r="V17" t="n">
-        <v>0.6296296296296297</v>
+        <v>0.7941176470588236</v>
       </c>
       <c r="W17" t="n">
-        <v>0.7916666666666666</v>
+        <v>0.6388888888888888</v>
       </c>
       <c r="X17" t="n">
+        <v>0.6111111111111112</v>
+      </c>
+      <c r="Y17" t="n">
         <v>0.7</v>
       </c>
-      <c r="Y17" t="n">
-        <v>0.6785714285714286</v>
-      </c>
       <c r="Z17" t="n">
-        <v>0.6</v>
+        <v>0.631578947368421</v>
       </c>
       <c r="AA17" t="n">
-        <v>0.3103448275862069</v>
-      </c>
-      <c r="AB17" t="inlineStr"/>
+        <v>0.5862068965517242</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>0.2564102564102564</v>
+      </c>
       <c r="AC17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>Lily Cheng</t>
+          <t>Rachel Chernos Lin</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.8444444444444444</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="C18" t="n">
-        <v>0.84</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="D18" t="n">
-        <v>0.8367346938775511</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="E18" t="n">
-        <v>0.7826086956521739</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>0.6923076923076923</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>0.8490566037735849</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="H18" t="n">
-        <v>0.8679245283018868</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="I18" t="n">
-        <v>0.8846153846153846</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="J18" t="n">
-        <v>0.8653846153846154</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="K18" t="n">
-        <v>0.8301886792452831</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="L18" t="n">
-        <v>0.8679245283018868</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="M18" t="n">
-        <v>0.8679245283018868</v>
+        <v>1</v>
       </c>
       <c r="N18" t="n">
-        <v>0.7959183673469388</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="O18" t="n">
-        <v>0.88</v>
+        <v>1</v>
       </c>
       <c r="P18" t="n">
-        <v>0.7551020408163265</v>
+        <v>1</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.8518518518518519</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="R18" t="n">
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>0.7169811320754718</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="T18" t="n">
-        <v>0.6122448979591837</v>
+        <v>1</v>
       </c>
       <c r="U18" t="n">
-        <v>0.6382978723404256</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="V18" t="n">
-        <v>0.5681818181818181</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="W18" t="n">
-        <v>0.6122448979591837</v>
+        <v>0.5</v>
       </c>
       <c r="X18" t="n">
-        <v>0.5862068965517242</v>
-      </c>
-      <c r="Y18" t="n">
-        <v>0.5294117647058824</v>
-      </c>
+        <v>0.6666666666666667</v>
+      </c>
+      <c r="Y18" t="inlineStr"/>
       <c r="Z18" t="n">
-        <v>0.45</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.3018867924528302</v>
+        <v>0.3333333333333334</v>
       </c>
       <c r="AB18" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="AC18" t="n">
-        <v>0.375</v>
-      </c>
+        <v>0.1428571428571429</v>
+      </c>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>Frances Nunziata</t>
+          <t>Lily Cheng</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.8085106382978724</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C19" t="n">
-        <v>0.7307692307692308</v>
+        <v>0.8305084745762712</v>
       </c>
       <c r="D19" t="n">
-        <v>0.8235294117647058</v>
+        <v>0.8275862068965517</v>
       </c>
       <c r="E19" t="n">
-        <v>0.75</v>
+        <v>0.7962962962962963</v>
       </c>
       <c r="F19" t="n">
-        <v>0.8780487804878049</v>
+        <v>0.7111111111111111</v>
       </c>
       <c r="G19" t="n">
-        <v>0.6909090909090909</v>
+        <v>0.8387096774193549</v>
       </c>
       <c r="H19" t="n">
-        <v>0.7407407407407407</v>
+        <v>0.8548387096774194</v>
       </c>
       <c r="I19" t="n">
-        <v>0.6851851851851851</v>
+        <v>0.8688524590163934</v>
       </c>
       <c r="J19" t="n">
-        <v>0.7407407407407407</v>
+        <v>0.8524590163934427</v>
       </c>
       <c r="K19" t="n">
-        <v>0.6727272727272727</v>
+        <v>0.8225806451612903</v>
       </c>
       <c r="L19" t="n">
-        <v>0.6727272727272727</v>
+        <v>0.8548387096774194</v>
       </c>
       <c r="M19" t="n">
-        <v>0.6727272727272727</v>
+        <v>0.8688524590163934</v>
       </c>
       <c r="N19" t="n">
-        <v>0.8431372549019608</v>
+        <v>0.864406779661017</v>
       </c>
       <c r="O19" t="n">
-        <v>0.6470588235294117</v>
+        <v>0.7818181818181819</v>
       </c>
       <c r="P19" t="n">
-        <v>0.7254901960784313</v>
+        <v>0.7719298245614035</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.8275862068965517</v>
+        <v>0.8055555555555556</v>
       </c>
       <c r="R19" t="n">
-        <v>0.7169811320754718</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="S19" t="n">
         <v>1</v>
       </c>
       <c r="T19" t="n">
-        <v>0.7450980392156863</v>
+        <v>0.7419354838709677</v>
       </c>
       <c r="U19" t="n">
-        <v>0.5510204081632653</v>
+        <v>0.6785714285714286</v>
       </c>
       <c r="V19" t="n">
-        <v>0.6739130434782609</v>
+        <v>0.6206896551724138</v>
       </c>
       <c r="W19" t="n">
-        <v>0.78</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="X19" t="n">
-        <v>0.6206896551724138</v>
+        <v>0.5961538461538461</v>
       </c>
       <c r="Y19" t="n">
-        <v>0.7169811320754718</v>
+        <v>0.5862068965517242</v>
       </c>
       <c r="Z19" t="n">
-        <v>0.7560975609756098</v>
+        <v>0.5166666666666666</v>
       </c>
       <c r="AA19" t="n">
-        <v>0.3454545454545455</v>
+        <v>0.4583333333333334</v>
       </c>
       <c r="AB19" t="n">
-        <v>1</v>
+        <v>0.2903225806451613</v>
       </c>
       <c r="AC19" t="n">
-        <v>1</v>
+        <v>0.375</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>0.375</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>Nick Mantas</t>
+          <t>Frances Nunziata</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.7674418604651163</v>
+        <v>0.8245614035087719</v>
       </c>
       <c r="C20" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.7580645161290323</v>
       </c>
       <c r="D20" t="n">
+        <v>0.8360655737704918</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.7894736842105263</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.8936170212765957</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.7230769230769231</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.765625</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.71875</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.765625</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.7076923076923076</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.7076923076923076</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.71875</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0.6885245901639344</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.8448275862068966</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0.7666666666666666</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.8205128205128205</v>
+      </c>
+      <c r="R20" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" t="n">
+        <v>0.7419354838709677</v>
+      </c>
+      <c r="T20" t="n">
+        <v>1</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0.5932203389830508</v>
+      </c>
+      <c r="V20" t="n">
         <v>0.75</v>
       </c>
-      <c r="E20" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0.8717948717948718</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0.6274509803921569</v>
-      </c>
-      <c r="H20" t="n">
+      <c r="W20" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="X20" t="n">
+        <v>0.6545454545454545</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>0.6206896551724138</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>0.6507936507936508</v>
+      </c>
+      <c r="AA20" t="n">
         <v>0.6799999999999999</v>
       </c>
-      <c r="I20" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0.6799999999999999</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0.607843137254902</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0.607843137254902</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0.607843137254902</v>
-      </c>
-      <c r="N20" t="n">
-        <v>0.7872340425531915</v>
-      </c>
-      <c r="O20" t="n">
-        <v>0.5957446808510638</v>
-      </c>
-      <c r="P20" t="n">
-        <v>0.6595744680851063</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>0.7037037037037037</v>
-      </c>
-      <c r="R20" t="n">
-        <v>0.6122448979591837</v>
-      </c>
-      <c r="S20" t="n">
-        <v>0.7450980392156863</v>
-      </c>
-      <c r="T20" t="n">
-        <v>1</v>
-      </c>
-      <c r="U20" t="n">
-        <v>0.7111111111111111</v>
-      </c>
-      <c r="V20" t="n">
-        <v>0.6904761904761905</v>
-      </c>
-      <c r="W20" t="n">
-        <v>0.7173913043478262</v>
-      </c>
-      <c r="X20" t="n">
-        <v>0.6296296296296297</v>
-      </c>
-      <c r="Y20" t="n">
-        <v>0.7551020408163265</v>
-      </c>
-      <c r="Z20" t="n">
-        <v>0.7105263157894737</v>
-      </c>
-      <c r="AA20" t="n">
-        <v>0.4117647058823529</v>
-      </c>
       <c r="AB20" t="n">
-        <v>0.875</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="AC20" t="n">
-        <v>0.875</v>
+        <v>1</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -20955,727 +21011,753 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.7380952380952381</v>
+        <v>0.7307692307692308</v>
       </c>
       <c r="C21" t="n">
-        <v>0.6304347826086957</v>
+        <v>0.6428571428571428</v>
       </c>
       <c r="D21" t="n">
+        <v>0.6181818181818182</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.6981132075471699</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.6511627906976745</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.6610169491525424</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.6724137931034483</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.6724137931034483</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.6379310344827587</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.6440677966101696</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0.6440677966101696</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.6551724137931034</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0.6545454545454545</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0.6226415094339622</v>
+      </c>
+      <c r="P21" t="n">
+        <v>0.6296296296296297</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0.6764705882352942</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="S21" t="n">
+        <v>0.6785714285714286</v>
+      </c>
+      <c r="T21" t="n">
+        <v>0.5932203389830508</v>
+      </c>
+      <c r="U21" t="n">
+        <v>1</v>
+      </c>
+      <c r="V21" t="n">
+        <v>0.6491228070175439</v>
+      </c>
+      <c r="W21" t="n">
+        <v>0.6666666666666667</v>
+      </c>
+      <c r="X21" t="n">
         <v>0.6</v>
       </c>
-      <c r="E21" t="n">
-        <v>0.6818181818181819</v>
-      </c>
-      <c r="F21" t="n">
-        <v>0.6486486486486487</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0.653061224489796</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0.6666666666666667</v>
-      </c>
-      <c r="I21" t="n">
-        <v>0.6666666666666667</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0.6326530612244898</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0.6326530612244898</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0.6326530612244898</v>
-      </c>
-      <c r="N21" t="n">
-        <v>0.6086956521739131</v>
-      </c>
-      <c r="O21" t="n">
-        <v>0.6444444444444444</v>
-      </c>
-      <c r="P21" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>0.7083333333333333</v>
-      </c>
-      <c r="R21" t="n">
-        <v>0.6382978723404256</v>
-      </c>
-      <c r="S21" t="n">
-        <v>0.5510204081632653</v>
-      </c>
-      <c r="T21" t="n">
-        <v>0.7111111111111111</v>
-      </c>
-      <c r="U21" t="n">
-        <v>1</v>
-      </c>
-      <c r="V21" t="n">
-        <v>0.5853658536585367</v>
-      </c>
-      <c r="W21" t="n">
-        <v>0.6170212765957447</v>
-      </c>
-      <c r="X21" t="n">
+      <c r="Y21" t="n">
         <v>0.6153846153846154</v>
       </c>
-      <c r="Y21" t="n">
-        <v>0.5319148936170213</v>
-      </c>
       <c r="Z21" t="n">
-        <v>0.5675675675675675</v>
+        <v>0.5263157894736843</v>
       </c>
       <c r="AA21" t="n">
-        <v>0.4081632653061225</v>
+        <v>0.5652173913043479</v>
       </c>
       <c r="AB21" t="n">
+        <v>0.3898305084745762</v>
+      </c>
+      <c r="AC21" t="n">
         <v>0.2857142857142857</v>
       </c>
-      <c r="AC21" t="n">
+      <c r="AD21" t="n">
         <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>Jon Burnside</t>
+          <t>James Pasternak</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.717948717948718</v>
+        <v>0.7115384615384616</v>
       </c>
       <c r="C22" t="n">
-        <v>0.6279069767441861</v>
+        <v>0.631578947368421</v>
       </c>
       <c r="D22" t="n">
-        <v>0.6428571428571428</v>
+        <v>0.6964285714285714</v>
       </c>
       <c r="E22" t="n">
         <v>0.6666666666666667</v>
       </c>
       <c r="F22" t="n">
-        <v>0.7272727272727273</v>
+        <v>0.7045454545454546</v>
       </c>
       <c r="G22" t="n">
-        <v>0.5652173913043479</v>
+        <v>0.6</v>
       </c>
       <c r="H22" t="n">
+        <v>0.6101694915254237</v>
+      </c>
+      <c r="I22" t="n">
         <v>0.6</v>
       </c>
-      <c r="I22" t="n">
-        <v>0.5555555555555556</v>
-      </c>
       <c r="J22" t="n">
-        <v>0.6222222222222222</v>
+        <v>0.6440677966101696</v>
       </c>
       <c r="K22" t="n">
-        <v>0.5652173913043479</v>
+        <v>0.5833333333333333</v>
       </c>
       <c r="L22" t="n">
-        <v>0.5434782608695652</v>
+        <v>0.5833333333333333</v>
       </c>
       <c r="M22" t="n">
-        <v>0.5434782608695652</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="N22" t="n">
-        <v>0.6904761904761905</v>
+        <v>0.5614035087719298</v>
       </c>
       <c r="O22" t="n">
+        <v>0.7547169811320755</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0.6071428571428572</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0.7941176470588236</v>
+      </c>
+      <c r="R22" t="n">
         <v>0.5714285714285714</v>
       </c>
-      <c r="P22" t="n">
-        <v>0.7142857142857143</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>0.6296296296296297</v>
-      </c>
-      <c r="R22" t="n">
-        <v>0.5681818181818181</v>
-      </c>
       <c r="S22" t="n">
-        <v>0.6739130434782609</v>
+        <v>0.6206896551724138</v>
       </c>
       <c r="T22" t="n">
-        <v>0.6904761904761905</v>
+        <v>0.75</v>
       </c>
       <c r="U22" t="n">
-        <v>0.5853658536585367</v>
+        <v>0.6491228070175439</v>
       </c>
       <c r="V22" t="n">
         <v>1</v>
       </c>
       <c r="W22" t="n">
-        <v>0.7804878048780488</v>
+        <v>0.6727272727272727</v>
       </c>
       <c r="X22" t="n">
-        <v>0.7</v>
+        <v>0.76</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.6590909090909092</v>
+        <v>0.8148148148148149</v>
       </c>
       <c r="Z22" t="n">
-        <v>0.631578947368421</v>
+        <v>0.6896551724137931</v>
       </c>
       <c r="AA22" t="n">
-        <v>0.4347826086956522</v>
+        <v>0.7708333333333334</v>
       </c>
       <c r="AB22" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.4166666666666666</v>
       </c>
       <c r="AC22" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.875</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>0.875</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>James Pasternak</t>
+          <t>Nick Mantas</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.6923076923076923</v>
       </c>
       <c r="C23" t="n">
-        <v>0.6170212765957447</v>
+        <v>0.6140350877192983</v>
       </c>
       <c r="D23" t="n">
-        <v>0.6956521739130435</v>
+        <v>0.6842105263157895</v>
       </c>
       <c r="E23" t="n">
+        <v>0.6923076923076923</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.8181818181818181</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.5833333333333333</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.6271186440677966</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.576271186440678</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.6271186440677966</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0.5666666666666667</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0.5666666666666667</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0.576271186440678</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0.5535714285714286</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0.7735849056603774</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.6181818181818182</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0.6388888888888888</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="S23" t="n">
+        <v>0.5789473684210527</v>
+      </c>
+      <c r="T23" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="U23" t="n">
         <v>0.6666666666666667</v>
       </c>
-      <c r="F23" t="n">
-        <v>0.736842105263158</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0.5800000000000001</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0.5918367346938775</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0.5800000000000001</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0.6326530612244898</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="N23" t="n">
-        <v>0.7391304347826086</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0.5319148936170213</v>
-      </c>
-      <c r="P23" t="n">
-        <v>0.5957446808510638</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-      <c r="R23" t="n">
-        <v>0.6122448979591837</v>
-      </c>
-      <c r="S23" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="T23" t="n">
-        <v>0.7173913043478262</v>
-      </c>
-      <c r="U23" t="n">
-        <v>0.6170212765957447</v>
-      </c>
       <c r="V23" t="n">
-        <v>0.7804878048780488</v>
+        <v>0.6727272727272727</v>
       </c>
       <c r="W23" t="n">
         <v>1</v>
       </c>
       <c r="X23" t="n">
-        <v>0.8148148148148149</v>
+        <v>0.7</v>
       </c>
       <c r="Y23" t="n">
-        <v>0.6875</v>
+        <v>0.6296296296296297</v>
       </c>
       <c r="Z23" t="n">
-        <v>0.7692307692307692</v>
+        <v>0.7586206896551724</v>
       </c>
       <c r="AA23" t="n">
-        <v>0.4399999999999999</v>
+        <v>0.7021276595744681</v>
       </c>
       <c r="AB23" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="AC23" t="n">
         <v>0.875</v>
       </c>
-      <c r="AC23" t="n">
+      <c r="AD23" t="n">
         <v>0.875</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>Jaye Robinson</t>
+          <t>Jon Burnside</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.6086956521739131</v>
+        <v>0.6666666666666667</v>
       </c>
       <c r="C24" t="n">
-        <v>0.5517241379310345</v>
+        <v>0.5961538461538461</v>
       </c>
       <c r="D24" t="n">
-        <v>0.5862068965517242</v>
+        <v>0.607843137254902</v>
       </c>
       <c r="E24" t="n">
-        <v>0.6538461538461539</v>
+        <v>0.6382978723404256</v>
       </c>
       <c r="F24" t="n">
-        <v>0.6818181818181819</v>
+        <v>0.7105263157894737</v>
       </c>
       <c r="G24" t="n">
-        <v>0.5517241379310345</v>
+        <v>0.5454545454545454</v>
       </c>
       <c r="H24" t="n">
-        <v>0.5172413793103448</v>
+        <v>0.5740740740740741</v>
       </c>
       <c r="I24" t="n">
-        <v>0.5862068965517242</v>
+        <v>0.537037037037037</v>
       </c>
       <c r="J24" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.5925925925925926</v>
       </c>
       <c r="K24" t="n">
-        <v>0.5172413793103448</v>
+        <v>0.5454545454545454</v>
       </c>
       <c r="L24" t="n">
-        <v>0.5517241379310345</v>
+        <v>0.5272727272727273</v>
       </c>
       <c r="M24" t="n">
-        <v>0.5517241379310345</v>
+        <v>0.537037037037037</v>
       </c>
       <c r="N24" t="n">
-        <v>0.6071428571428572</v>
+        <v>0.5490196078431373</v>
       </c>
       <c r="O24" t="n">
-        <v>0.5</v>
+        <v>0.6734693877551021</v>
       </c>
       <c r="P24" t="n">
-        <v>0.5357142857142857</v>
+        <v>0.6799999999999999</v>
       </c>
       <c r="Q24" t="n">
+        <v>0.6111111111111112</v>
+      </c>
+      <c r="R24" t="n">
+        <v>0.6666666666666667</v>
+      </c>
+      <c r="S24" t="n">
+        <v>0.5961538461538461</v>
+      </c>
+      <c r="T24" t="n">
+        <v>0.6545454545454545</v>
+      </c>
+      <c r="U24" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="V24" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="W24" t="n">
         <v>0.7</v>
       </c>
-      <c r="R24" t="n">
-        <v>0.5862068965517242</v>
-      </c>
-      <c r="S24" t="n">
-        <v>0.6206896551724138</v>
-      </c>
-      <c r="T24" t="n">
-        <v>0.6296296296296297</v>
-      </c>
-      <c r="U24" t="n">
-        <v>0.6153846153846154</v>
-      </c>
-      <c r="V24" t="n">
+      <c r="X24" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y24" t="n">
         <v>0.7</v>
       </c>
-      <c r="W24" t="n">
-        <v>0.8148148148148149</v>
-      </c>
-      <c r="X24" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y24" t="n">
-        <v>0.6551724137931034</v>
-      </c>
       <c r="Z24" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.679245283018868</v>
       </c>
       <c r="AA24" t="n">
-        <v>0.5172413793103448</v>
+        <v>0.6304347826086957</v>
       </c>
       <c r="AB24" t="n">
-        <v>0.5</v>
+        <v>0.4545454545454546</v>
       </c>
       <c r="AC24" t="n">
-        <v>0.5</v>
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>0.7142857142857143</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>Brad Bradford</t>
+          <t>Jaye Robinson</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.5777777777777777</v>
+        <v>0.6086956521739131</v>
       </c>
       <c r="C25" t="n">
-        <v>0.5490196078431373</v>
+        <v>0.5517241379310345</v>
       </c>
       <c r="D25" t="n">
-        <v>0.64</v>
+        <v>0.5862068965517242</v>
       </c>
       <c r="E25" t="n">
-        <v>0.6170212765957447</v>
+        <v>0.6538461538461539</v>
       </c>
       <c r="F25" t="n">
-        <v>0.6829268292682926</v>
+        <v>0.6818181818181819</v>
       </c>
       <c r="G25" t="n">
-        <v>0.5094339622641509</v>
+        <v>0.5517241379310345</v>
       </c>
       <c r="H25" t="n">
-        <v>0.5576923076923077</v>
+        <v>0.5172413793103448</v>
       </c>
       <c r="I25" t="n">
+        <v>0.5862068965517242</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0.5172413793103448</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0.5517241379310345</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0.5517241379310345</v>
+      </c>
+      <c r="N25" t="n">
         <v>0.5</v>
       </c>
-      <c r="J25" t="n">
-        <v>0.5576923076923077</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0.4905660377358491</v>
-      </c>
-      <c r="L25" t="n">
-        <v>0.4905660377358491</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0.4905660377358491</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0.7142857142857143</v>
-      </c>
       <c r="O25" t="n">
-        <v>0.4693877551020408</v>
+        <v>0.6071428571428572</v>
       </c>
       <c r="P25" t="n">
-        <v>0.5918367346938775</v>
+        <v>0.5357142857142857</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.6785714285714286</v>
-      </c>
-      <c r="R25" t="n">
-        <v>0.5294117647058824</v>
-      </c>
+        <v>0.7</v>
+      </c>
+      <c r="R25" t="inlineStr"/>
       <c r="S25" t="n">
-        <v>0.7169811320754718</v>
+        <v>0.5862068965517242</v>
       </c>
       <c r="T25" t="n">
-        <v>0.7551020408163265</v>
+        <v>0.6206896551724138</v>
       </c>
       <c r="U25" t="n">
-        <v>0.5319148936170213</v>
+        <v>0.6153846153846154</v>
       </c>
       <c r="V25" t="n">
-        <v>0.6590909090909092</v>
+        <v>0.8148148148148149</v>
       </c>
       <c r="W25" t="n">
-        <v>0.6875</v>
+        <v>0.6296296296296297</v>
       </c>
       <c r="X25" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z25" t="n">
         <v>0.6551724137931034</v>
       </c>
-      <c r="Y25" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z25" t="n">
-        <v>0.7</v>
-      </c>
       <c r="AA25" t="n">
-        <v>0.5471698113207547</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="AB25" t="n">
-        <v>0.875</v>
+        <v>0.5172413793103448</v>
       </c>
       <c r="AC25" t="n">
-        <v>0.875</v>
+        <v>0.5</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>Vincent Crisanti</t>
+          <t>Brad Bradford</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.5151515151515151</v>
+        <v>0.5454545454545454</v>
       </c>
       <c r="C26" t="n">
-        <v>0.4736842105263158</v>
+        <v>0.5245901639344263</v>
       </c>
       <c r="D26" t="n">
-        <v>0.5526315789473684</v>
+        <v>0.6</v>
       </c>
       <c r="E26" t="n">
-        <v>0.5277777777777778</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="F26" t="n">
-        <v>0.6666666666666667</v>
+        <v>0.6382978723404256</v>
       </c>
       <c r="G26" t="n">
-        <v>0.4146341463414634</v>
+        <v>0.4920634920634921</v>
       </c>
       <c r="H26" t="n">
-        <v>0.4878048780487805</v>
+        <v>0.532258064516129</v>
       </c>
       <c r="I26" t="n">
-        <v>0.4146341463414634</v>
+        <v>0.4838709677419355</v>
       </c>
       <c r="J26" t="n">
-        <v>0.475</v>
+        <v>0.532258064516129</v>
       </c>
       <c r="K26" t="n">
-        <v>0.4146341463414634</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="L26" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="M26" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.467741935483871</v>
       </c>
       <c r="N26" t="n">
+        <v>0.4576271186440678</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0.6964285714285714</v>
+      </c>
+      <c r="P26" t="n">
+        <v>0.5517241379310345</v>
+      </c>
+      <c r="Q26" t="n">
         <v>0.631578947368421</v>
       </c>
-      <c r="O26" t="n">
-        <v>0.3783783783783784</v>
-      </c>
-      <c r="P26" t="n">
-        <v>0.5526315789473684</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>0.6</v>
-      </c>
       <c r="R26" t="n">
-        <v>0.45</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="S26" t="n">
-        <v>0.7560975609756098</v>
+        <v>0.5166666666666666</v>
       </c>
       <c r="T26" t="n">
-        <v>0.7105263157894737</v>
+        <v>0.6507936507936508</v>
       </c>
       <c r="U26" t="n">
-        <v>0.5675675675675675</v>
+        <v>0.5263157894736843</v>
       </c>
       <c r="V26" t="n">
-        <v>0.631578947368421</v>
+        <v>0.6896551724137931</v>
       </c>
       <c r="W26" t="n">
-        <v>0.7692307692307692</v>
+        <v>0.7586206896551724</v>
       </c>
       <c r="X26" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.679245283018868</v>
       </c>
       <c r="Y26" t="n">
-        <v>0.7</v>
+        <v>0.6551724137931034</v>
       </c>
       <c r="Z26" t="n">
         <v>1</v>
       </c>
       <c r="AA26" t="n">
-        <v>0.6097560975609756</v>
+        <v>0.7346938775510203</v>
       </c>
       <c r="AB26" t="n">
-        <v>1</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="AC26" t="n">
-        <v>1</v>
+        <v>0.875</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>0.875</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>Stephen Holyday</t>
+          <t>Vincent Crisanti</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.148936170212766</v>
+        <v>0.5</v>
       </c>
       <c r="C27" t="n">
-        <v>0.1730769230769231</v>
+        <v>0.4680851063829787</v>
       </c>
       <c r="D27" t="n">
-        <v>0.2156862745098039</v>
+        <v>0.5319148936170213</v>
       </c>
       <c r="E27" t="n">
-        <v>0.2708333333333334</v>
+        <v>0.5</v>
       </c>
       <c r="F27" t="n">
-        <v>0.2682926829268293</v>
+        <v>0.6</v>
       </c>
       <c r="G27" t="n">
-        <v>0.1454545454545455</v>
+        <v>0.42</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2407407407407407</v>
+        <v>0.48</v>
       </c>
       <c r="I27" t="n">
-        <v>0.1666666666666666</v>
+        <v>0.42</v>
       </c>
       <c r="J27" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.4693877551020408</v>
       </c>
       <c r="K27" t="n">
-        <v>0.2</v>
+        <v>0.42</v>
       </c>
       <c r="L27" t="n">
-        <v>0.1636363636363637</v>
+        <v>0.4</v>
       </c>
       <c r="M27" t="n">
-        <v>0.1636363636363637</v>
+        <v>0.3877551020408163</v>
       </c>
       <c r="N27" t="n">
-        <v>0.2745098039215687</v>
+        <v>0.3913043478260869</v>
       </c>
       <c r="O27" t="n">
-        <v>0.196078431372549</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="P27" t="n">
-        <v>0.2941176470588235</v>
+        <v>0.5217391304347826</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.3103448275862069</v>
+        <v>0.5862068965517242</v>
       </c>
       <c r="R27" t="n">
-        <v>0.3018867924528302</v>
+        <v>0.3333333333333334</v>
       </c>
       <c r="S27" t="n">
-        <v>0.3454545454545455</v>
+        <v>0.4583333333333334</v>
       </c>
       <c r="T27" t="n">
-        <v>0.4117647058823529</v>
+        <v>0.6799999999999999</v>
       </c>
       <c r="U27" t="n">
-        <v>0.4081632653061225</v>
+        <v>0.5652173913043479</v>
       </c>
       <c r="V27" t="n">
-        <v>0.4347826086956522</v>
+        <v>0.7708333333333334</v>
       </c>
       <c r="W27" t="n">
-        <v>0.4399999999999999</v>
+        <v>0.7021276595744681</v>
       </c>
       <c r="X27" t="n">
-        <v>0.5172413793103448</v>
+        <v>0.6304347826086957</v>
       </c>
       <c r="Y27" t="n">
-        <v>0.5471698113207547</v>
+        <v>0.5789473684210527</v>
       </c>
       <c r="Z27" t="n">
-        <v>0.6097560975609756</v>
+        <v>0.7346938775510203</v>
       </c>
       <c r="AA27" t="n">
         <v>1</v>
       </c>
       <c r="AB27" t="n">
-        <v>0.375</v>
+        <v>0.6</v>
       </c>
       <c r="AC27" t="n">
-        <v>0.375</v>
+        <v>1</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>John Tory</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
+          <t>Stephen Holyday</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0.1228070175438597</v>
+      </c>
       <c r="C28" t="n">
-        <v>0.5</v>
+        <v>0.1451612903225806</v>
       </c>
       <c r="D28" t="n">
-        <v>0.875</v>
+        <v>0.180327868852459</v>
       </c>
       <c r="E28" t="n">
-        <v>0.625</v>
+        <v>0.2280701754385965</v>
       </c>
       <c r="F28" t="n">
-        <v>0.875</v>
+        <v>0.2340425531914894</v>
       </c>
       <c r="G28" t="n">
+        <v>0.1230769230769231</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.203125</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0.140625</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.1692307692307692</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0.1384615384615384</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0.140625</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0.1639344262295082</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0.2586206896551724</v>
+      </c>
+      <c r="P28" t="n">
         <v>0.25</v>
       </c>
-      <c r="H28" t="n">
+      <c r="Q28" t="n">
+        <v>0.2564102564102564</v>
+      </c>
+      <c r="R28" t="n">
+        <v>0.1428571428571429</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0.2903225806451613</v>
+      </c>
+      <c r="T28" t="n">
+        <v>0.3076923076923077</v>
+      </c>
+      <c r="U28" t="n">
+        <v>0.3898305084745762</v>
+      </c>
+      <c r="V28" t="n">
+        <v>0.4166666666666666</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="X28" t="n">
+        <v>0.4545454545454546</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>0.5172413793103448</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>0.5555555555555556</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="AB28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC28" t="n">
         <v>0.375</v>
       </c>
-      <c r="I28" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="J28" t="n">
-        <v>0.4285714285714286</v>
-      </c>
-      <c r="K28" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="L28" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M28" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="N28" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="O28" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="P28" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="n">
+      <c r="AD28" t="n">
         <v>0.375</v>
-      </c>
-      <c r="S28" t="n">
-        <v>1</v>
-      </c>
-      <c r="T28" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="U28" t="n">
-        <v>0.2857142857142857</v>
-      </c>
-      <c r="V28" t="n">
-        <v>0.7142857142857143</v>
-      </c>
-      <c r="W28" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="X28" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Y28" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="Z28" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA28" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="AB28" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC28" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>Gary Crawford</t>
+          <t>John Tory</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -21713,49 +21795,138 @@
         <v>0.25</v>
       </c>
       <c r="N29" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="O29" t="n">
         <v>0.875</v>
-      </c>
-      <c r="O29" t="n">
-        <v>0.25</v>
       </c>
       <c r="P29" t="n">
         <v>0.625</v>
       </c>
       <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="n">
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="n">
         <v>0.375</v>
       </c>
-      <c r="S29" t="n">
-        <v>1</v>
-      </c>
       <c r="T29" t="n">
-        <v>0.875</v>
+        <v>1</v>
       </c>
       <c r="U29" t="n">
         <v>0.2857142857142857</v>
       </c>
       <c r="V29" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.875</v>
       </c>
       <c r="W29" t="n">
         <v>0.875</v>
       </c>
       <c r="X29" t="n">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="Y29" t="n">
         <v>0.5</v>
       </c>
-      <c r="Y29" t="n">
+      <c r="Z29" t="n">
         <v>0.875</v>
       </c>
-      <c r="Z29" t="n">
-        <v>1</v>
-      </c>
       <c r="AA29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB29" t="n">
         <v>0.375</v>
       </c>
-      <c r="AB29" t="n">
-        <v>1</v>
-      </c>
       <c r="AC29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>Gary Crawford</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.4285714285714286</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="P30" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="T30" t="n">
+        <v>1</v>
+      </c>
+      <c r="U30" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="V30" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="W30" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="X30" t="n">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AA30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB30" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD30" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>